<commit_message>
Fix SPD03015 title band formatting
</commit_message>
<xml_diff>
--- a/templates/spd03015_irm_sap_template.xlsx
+++ b/templates/spd03015_irm_sap_template.xlsx
@@ -157,7 +157,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -194,8 +194,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000338D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00338D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -335,11 +345,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="43" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -533,6 +574,42 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -968,7 +1045,7 @@
       <c r="AI1" s="1" t="n"/>
     </row>
     <row r="2" outlineLevel="1" ht="50" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="84" t="inlineStr">
         <is>
           <t>kpmg    Inventory cost variance
  allocation (standard
@@ -977,60 +1054,85 @@
 存货成本差异分摊（标准成本法）— 重新计算</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="n"/>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="n"/>
-      <c r="M2" s="7" t="n"/>
-      <c r="R2" s="1" t="n"/>
+      <c r="B2" s="85" t="n"/>
+      <c r="C2" s="85" t="n"/>
+      <c r="D2" s="85" t="n"/>
+      <c r="E2" s="85" t="n"/>
+      <c r="F2" s="86" t="n"/>
+      <c r="G2" s="86" t="n"/>
+      <c r="H2" s="86" t="n"/>
+      <c r="I2" s="87" t="n"/>
+      <c r="J2" s="87" t="n"/>
+      <c r="K2" s="87" t="n"/>
+      <c r="L2" s="87" t="n"/>
+      <c r="M2" s="87" t="n"/>
+      <c r="N2" s="88" t="n"/>
+      <c r="O2" s="88" t="n"/>
+      <c r="P2" s="88" t="n"/>
+      <c r="Q2" s="88" t="n"/>
+      <c r="R2" s="89" t="n"/>
+      <c r="S2" s="88" t="n"/>
+      <c r="T2" s="88" t="n"/>
+      <c r="U2" s="88" t="n"/>
+      <c r="V2" s="88" t="n"/>
+      <c r="W2" s="88" t="n"/>
+      <c r="X2" s="88" t="n"/>
+      <c r="Y2" s="88" t="n"/>
+      <c r="Z2" s="88" t="n"/>
+      <c r="AA2" s="88" t="n"/>
+      <c r="AB2" s="88" t="n"/>
+      <c r="AC2" s="88" t="n"/>
+      <c r="AD2" s="88" t="n"/>
+      <c r="AE2" s="88" t="n"/>
+      <c r="AF2" s="88" t="n"/>
+      <c r="AG2" s="88" t="n"/>
+      <c r="AH2" s="88" t="n"/>
+      <c r="AI2" s="88" t="n"/>
+      <c r="AJ2" s="88" t="n"/>
+      <c r="AK2" s="88" t="n"/>
     </row>
     <row r="3" outlineLevel="1" ht="14.5" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="90" t="inlineStr">
         <is>
           <t>(This substantive procedure template is used to test the inventory cost variance allocation) (本实质性程序模板用于测试存货成本差异分摊)</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
-      <c r="L3" s="9" t="n"/>
-      <c r="M3" s="9" t="n"/>
-      <c r="N3" s="8" t="n"/>
-      <c r="O3" s="8" t="n"/>
-      <c r="P3" s="1" t="n"/>
-      <c r="Q3" s="1" t="n"/>
-      <c r="R3" s="1" t="n"/>
-      <c r="S3" s="1" t="n"/>
-      <c r="T3" s="1" t="n"/>
-      <c r="U3" s="1" t="n"/>
-      <c r="V3" s="1" t="n"/>
-      <c r="W3" s="1" t="n"/>
-      <c r="X3" s="1" t="n"/>
-      <c r="Y3" s="1" t="n"/>
-      <c r="Z3" s="1" t="n"/>
-      <c r="AA3" s="1" t="n"/>
-      <c r="AB3" s="1" t="n"/>
-      <c r="AC3" s="1" t="n"/>
-      <c r="AD3" s="1" t="n"/>
-      <c r="AE3" s="1" t="n"/>
-      <c r="AF3" s="1" t="n"/>
-      <c r="AG3" s="3" t="n"/>
-      <c r="AH3" s="1" t="n"/>
-      <c r="AI3" s="1" t="n"/>
+      <c r="B3" s="90" t="n"/>
+      <c r="C3" s="90" t="n"/>
+      <c r="D3" s="90" t="n"/>
+      <c r="E3" s="90" t="n"/>
+      <c r="F3" s="90" t="n"/>
+      <c r="G3" s="90" t="n"/>
+      <c r="H3" s="90" t="n"/>
+      <c r="I3" s="91" t="n"/>
+      <c r="J3" s="91" t="n"/>
+      <c r="K3" s="91" t="n"/>
+      <c r="L3" s="91" t="n"/>
+      <c r="M3" s="91" t="n"/>
+      <c r="N3" s="90" t="n"/>
+      <c r="O3" s="90" t="n"/>
+      <c r="P3" s="89" t="n"/>
+      <c r="Q3" s="89" t="n"/>
+      <c r="R3" s="89" t="n"/>
+      <c r="S3" s="89" t="n"/>
+      <c r="T3" s="89" t="n"/>
+      <c r="U3" s="89" t="n"/>
+      <c r="V3" s="89" t="n"/>
+      <c r="W3" s="89" t="n"/>
+      <c r="X3" s="89" t="n"/>
+      <c r="Y3" s="89" t="n"/>
+      <c r="Z3" s="89" t="n"/>
+      <c r="AA3" s="89" t="n"/>
+      <c r="AB3" s="89" t="n"/>
+      <c r="AC3" s="89" t="n"/>
+      <c r="AD3" s="89" t="n"/>
+      <c r="AE3" s="89" t="n"/>
+      <c r="AF3" s="89" t="n"/>
+      <c r="AG3" s="92" t="n"/>
+      <c r="AH3" s="89" t="n"/>
+      <c r="AI3" s="89" t="n"/>
+      <c r="AJ3" s="88" t="n"/>
+      <c r="AK3" s="88" t="n"/>
     </row>
     <row r="4" outlineLevel="1">
       <c r="A4" s="10" t="n"/>
@@ -1279,18 +1381,26 @@
 基于生产报告/明细账</t>
         </is>
       </c>
+      <c r="C16" s="82" t="n"/>
+      <c r="D16" s="82" t="n"/>
+      <c r="E16" s="82" t="n"/>
+      <c r="F16" s="82" t="n"/>
+      <c r="G16" s="83" t="n"/>
       <c r="H16" s="35" t="inlineStr">
         <is>
           <t>Supporting document
 相关文件</t>
         </is>
       </c>
+      <c r="I16" s="83" t="n"/>
       <c r="J16" s="36" t="n"/>
       <c r="K16" s="36" t="inlineStr">
         <is>
           <t>4 = Reperform the calculation</t>
         </is>
       </c>
+      <c r="L16" s="82" t="n"/>
+      <c r="M16" s="82" t="n"/>
       <c r="N16" s="37" t="n"/>
       <c r="O16" s="38" t="inlineStr">
         <is>
@@ -1298,6 +1408,8 @@
 测试步骤</t>
         </is>
       </c>
+      <c r="P16" s="82" t="n"/>
+      <c r="Q16" s="83" t="n"/>
       <c r="R16" s="39" t="n"/>
       <c r="AJ16" s="40" t="n"/>
     </row>
@@ -1997,961 +2109,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
     <row r="986">
       <c r="A986" s="40" t="inlineStr">
         <is>
@@ -3026,14 +2183,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="Y10" s="70" t="inlineStr">
         <is>
@@ -3094,39 +2243,6 @@
         <v>-15066.9</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="69" t="inlineStr">
         <is>
@@ -3134,12 +2250,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="Y56" s="70" t="inlineStr">
         <is>
@@ -3205,43 +2315,6 @@
         <v>-227.55</v>
       </c>
     </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
     <row r="99">
       <c r="A99" s="69" t="inlineStr">
         <is>
@@ -3249,23 +2322,6 @@
         </is>
       </c>
     </row>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
     <row r="117">
       <c r="Y117" s="70" t="inlineStr">
         <is>
@@ -3326,31 +2382,6 @@
         <v>128</v>
       </c>
     </row>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
     <row r="148">
       <c r="A148" s="69" t="inlineStr">
         <is>
@@ -3358,24 +2389,6 @@
         </is>
       </c>
     </row>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
     <row r="167">
       <c r="Y167" s="70" t="inlineStr">
         <is>
@@ -3436,30 +2449,6 @@
         <v>-3376.38</v>
       </c>
     </row>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
     <row r="197">
       <c r="A197" s="69" t="inlineStr">
         <is>
@@ -3467,21 +2456,6 @@
         </is>
       </c>
     </row>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
     <row r="213">
       <c r="Y213" s="70" t="inlineStr">
         <is>

</xml_diff>